<commit_message>
modify detail to assetinfo
</commit_message>
<xml_diff>
--- a/src/src/main/resources/inventoryOrder.xlsx
+++ b/src/src/main/resources/inventoryOrder.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet 1 - 盘点工单" sheetId="1" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -14,7 +14,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Jiang, Jason (MOHLTC)</author>
+    <author>Zongbo Zhou</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0">
@@ -25,12 +25,12 @@
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
           </rPr>
-          <t>Jiang, Jason (MOHLTC):
-tie:form(name="listInventoryOrder" length="8" headerLength="0" footerLength="0")</t>
+          <t>Zongbo Zhou:
+tie:form(name="listInventoryOrder" length="7" headerLength="0" footerLength="0")</t>
         </r>
       </text>
     </comment>
-    <comment ref="A2" authorId="0">
+    <comment ref="A3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -38,12 +38,12 @@
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
           </rPr>
-          <t>Jiang, Jason (MOHLTC):
-tie:each(items="listInventoryOrder", var="inventoryOrder", length="7" allowAdd="False")</t>
+          <t>Zongbo Zhou:
+tie:each(items="listInventoryOrder", var="order", length="5" allowAdd="False")</t>
         </r>
       </text>
     </comment>
-    <comment ref="B2" authorId="0">
+    <comment ref="A4" authorId="0">
       <text>
         <r>
           <rPr>
@@ -51,34 +51,8 @@
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
           </rPr>
-          <t>Jiang, Jason (MOHLTC):
-Department name</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B4" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color indexed="8"/>
-            <rFont val="Helvetica Neue"/>
-          </rPr>
-          <t>Jiang, Jason (MOHLTC):
-${department.headAccount}</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A8" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color indexed="8"/>
-            <rFont val="Helvetica Neue"/>
-          </rPr>
-          <t>Jiang, Jason (MOHLTC):
-tie:each(items="inventoryOrder.inventoryOrderDetailList", var="detail", length="1" allowAdd="False")</t>
+          <t>Zongbo Zhou:
+tie:each(items="order.inventoryOrderDetailList", var="detail", length="4" allowAdd="False")</t>
         </r>
       </text>
     </comment>
@@ -87,87 +61,72 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="27">
-  <si>
-    <t>InventoryOrder</t>
-  </si>
-  <si>
-    <t>Name:</t>
-  </si>
-  <si>
-    <t>${inventoryOrder.name}</t>
-  </si>
-  <si>
-    <t>开始时间:</t>
-  </si>
-  <si>
-    <t>${inventoryOrder.startTime}</t>
-  </si>
-  <si>
-    <t>结束时间:</t>
-  </si>
-  <si>
-    <t>${inventoryOrder.endTime}</t>
-  </si>
-  <si>
-    <t>是否完成:</t>
-  </si>
-  <si>
-    <t>${inventoryOrder.isFinished}</t>
-  </si>
-  <si>
-    <t>设备编号</t>
-  </si>
-  <si>
-    <t>设备组名</t>
-  </si>
-  <si>
-    <t>备注</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="22">
+  <si>
+    <t>盘点工单</t>
+  </si>
+  <si>
+    <t>计划开始时间</t>
+  </si>
+  <si>
+    <t>${order.planStartTime}</t>
+  </si>
+  <si>
+    <t>计划结束时间</t>
+  </si>
+  <si>
+    <t>${order.planEndTime}</t>
   </si>
   <si>
     <t>状态</t>
   </si>
   <si>
+    <t>${order.isFinished}</t>
+  </si>
+  <si>
+    <t>科室名称</t>
+  </si>
+  <si>
     <t>设备名称</t>
   </si>
   <si>
     <t>设备型号</t>
   </si>
   <si>
-    <t>功能等级</t>
-  </si>
-  <si>
-    <t>制造商</t>
-  </si>
-  <si>
-    <t>维修商</t>
-  </si>
-  <si>
-    <t>${detail.departNum}</t>
-  </si>
-  <si>
-    <t>${detail.assetGroupName}</t>
-  </si>
-  <si>
-    <t>${detail.comment}</t>
-  </si>
-  <si>
-    <t>${detail.status}</t>
+    <t>设备序列号</t>
+  </si>
+  <si>
+    <t>设备财产号</t>
+  </si>
+  <si>
+    <t>使用科室</t>
+  </si>
+  <si>
+    <t>使用责任人</t>
+  </si>
+  <si>
+    <t>资产状态</t>
   </si>
   <si>
     <t>${detail.assetInfo.name}</t>
   </si>
   <si>
-    <t>${detail.assetInfo.functionType}</t>
-  </si>
-  <si>
-    <t>${detail.assetInfo.functionGrade}</t>
-  </si>
-  <si>
-    <t>${detail.assetInfo.manufacture}</t>
-  </si>
-  <si>
-    <t>${detail.assetInfo.maitanance}</t>
+    <t>${detail.assetInfo.departNum}</t>
+  </si>
+  <si>
+    <t>${detail.assetInfo.serialNum}</t>
+  </si>
+  <si>
+    <t>${detail.assetInfo.financingNum}</t>
+  </si>
+  <si>
+    <t>${detail.assetInfo.clinicalDeptName}</t>
+  </si>
+  <si>
+    <t>${detail.assetInfo.clinicalOwnerName}</t>
+  </si>
+  <si>
+    <t>${detail.assetInfo.status}</t>
   </si>
 </sst>
 </file>
@@ -177,7 +136,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -198,54 +157,6 @@
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Monaco"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Georgia"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="16"/>
-      <color indexed="11"/>
-      <name val="Cambria"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="10"/>
-      <color indexed="11"/>
-      <name val="Georgia"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="13"/>
-      <name val="Georgia"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color indexed="14"/>
-      <name val="Georgia"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="8"/>
-      <color indexed="8"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color indexed="9"/>
-      <name val="Georgia"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="8"/>
-      <name val="Georgia"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -262,53 +173,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="12"/>
+        <fgColor indexed="11"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="11"/>
+        <fgColor indexed="12"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="10"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -322,42 +202,8 @@
       <top style="thin">
         <color indexed="10"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
+      <bottom style="thin">
         <color indexed="10"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color indexed="9"/>
       </bottom>
       <diagonal/>
     </border>
@@ -365,12 +211,14 @@
       <left style="thin">
         <color indexed="10"/>
       </left>
-      <right/>
-      <top style="thick">
-        <color indexed="9"/>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="thin">
+        <color indexed="10"/>
       </top>
-      <bottom style="thick">
-        <color indexed="9"/>
+      <bottom style="thin">
+        <color indexed="13"/>
       </bottom>
       <diagonal/>
     </border>
@@ -378,133 +226,12 @@
       <left style="thin">
         <color indexed="10"/>
       </left>
-      <right/>
-      <top style="thick">
-        <color indexed="9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="9"/>
-      </left>
-      <right style="thin">
-        <color indexed="9"/>
-      </right>
-      <top style="thin">
-        <color indexed="9"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="9"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="13"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="10"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="9"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="9"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top style="thin">
-        <color indexed="9"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="10"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="10"/>
       </bottom>
@@ -516,122 +243,44 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="4" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="18" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="18" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="19" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="18" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -652,11 +301,10 @@
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
       <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ff666699"/>
-      <rgbColor rgb="ffc0c0c0"/>
-      <rgbColor rgb="ff333333"/>
-      <rgbColor rgb="ff865357"/>
+      <rgbColor rgb="ffa5a5a5"/>
+      <rgbColor rgb="ffdddddd"/>
+      <rgbColor rgb="ffbdc0bf"/>
+      <rgbColor rgb="ff3f3f3f"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1725,188 +1373,130 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
-  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="13.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="27.6094" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.9688" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.7891" style="1" customWidth="1"/>
-    <col min="4" max="4" width="27.7578" style="1" customWidth="1"/>
-    <col min="5" max="5" width="34.2891" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.3516" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.3516" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.3516" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.3516" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.3516" style="1" customWidth="1"/>
     <col min="6" max="6" width="16.3516" style="1" customWidth="1"/>
     <col min="7" max="7" width="16.3516" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.3516" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.3516" style="1" customWidth="1"/>
-    <col min="10" max="10" width="16.3516" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16.3516" style="1" customWidth="1"/>
-    <col min="12" max="256" width="16.3516" style="1" customWidth="1"/>
+    <col min="8" max="256" width="16.3516" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.65" customHeight="1">
+    <row r="1" ht="16.95" customHeight="1">
       <c r="A1" s="2"/>
-      <c r="B1" t="s" s="3">
+      <c r="B1" s="2"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" ht="20.35" customHeight="1">
+      <c r="A2" t="s" s="4">
         <v>0</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
     </row>
-    <row r="2" ht="20.25" customHeight="1">
-      <c r="A2" t="s" s="8">
+    <row r="3" ht="38.25" customHeight="1">
+      <c r="A3" t="s" s="6">
         <v>1</v>
       </c>
-      <c r="B2" t="s" s="9">
+      <c r="B3" t="s" s="6">
         <v>2</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="13"/>
+      <c r="C3" t="s" s="6">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s" s="6">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s" s="6">
+        <v>5</v>
+      </c>
+      <c r="F3" t="s" s="6">
+        <v>6</v>
+      </c>
+      <c r="G3" s="7"/>
     </row>
-    <row r="3" ht="20.25" customHeight="1">
-      <c r="A3" t="s" s="14">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s" s="15">
-        <v>4</v>
-      </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="17"/>
+    <row r="4" ht="14.25" customHeight="1">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
     </row>
-    <row r="4" ht="32.05" customHeight="1">
-      <c r="A4" t="s" s="18">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s" s="19">
-        <v>6</v>
-      </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="21"/>
+    <row r="5" ht="16.35" customHeight="1">
+      <c r="A5" t="s" s="10">
+        <v>7</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
     </row>
-    <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" t="s" s="22">
-        <v>7</v>
-      </c>
-      <c r="B5" t="s" s="19">
+    <row r="6" ht="16.35" customHeight="1">
+      <c r="A6" t="s" s="12">
         <v>8</v>
       </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="24"/>
+      <c r="B6" t="s" s="12">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s" s="12">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s" s="12">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s" s="12">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s" s="12">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s" s="12">
+        <v>14</v>
+      </c>
     </row>
-    <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" s="25"/>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="26"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="26"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="28"/>
-    </row>
-    <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" t="s" s="29">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s" s="29">
-        <v>10</v>
-      </c>
-      <c r="C7" t="s" s="29">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s" s="29">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s" s="29">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s" s="29">
-        <v>14</v>
-      </c>
-      <c r="G7" t="s" s="29">
+    <row r="7" ht="38.05" customHeight="1">
+      <c r="A7" t="s" s="12">
         <v>15</v>
       </c>
-      <c r="H7" t="s" s="29">
+      <c r="B7" t="s" s="12">
         <v>16</v>
       </c>
-      <c r="I7" t="s" s="29">
+      <c r="C7" t="s" s="12">
         <v>17</v>
       </c>
-      <c r="J7" s="30"/>
-      <c r="K7" s="31"/>
-    </row>
-    <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" t="s" s="32">
+      <c r="D7" t="s" s="12">
         <v>18</v>
       </c>
-      <c r="B8" t="s" s="33">
+      <c r="E7" t="s" s="12">
         <v>19</v>
       </c>
-      <c r="C8" t="s" s="34">
+      <c r="F7" t="s" s="12">
         <v>20</v>
       </c>
-      <c r="D8" t="s" s="35">
+      <c r="G7" t="s" s="12">
         <v>21</v>
       </c>
-      <c r="E8" t="s" s="32">
-        <v>22</v>
-      </c>
-      <c r="F8" t="s" s="36">
-        <v>23</v>
-      </c>
-      <c r="G8" t="s" s="36">
-        <v>24</v>
-      </c>
-      <c r="H8" t="s" s="36">
-        <v>25</v>
-      </c>
-      <c r="I8" t="s" s="36">
-        <v>26</v>
-      </c>
-      <c r="J8" s="37"/>
-      <c r="K8" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B4:G4"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>